<commit_message>
updated reg.xlsx to Sept 11 2025
</commit_message>
<xml_diff>
--- a/BOND_EQT/reg.xlsx
+++ b/BOND_EQT/reg.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c060ac0a7f9c7ae2/main/CRAMC_Desktop/EU/BOND_EQT/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="80" documentId="11_F25DC773A252ABDACC1048DAA15A48A85ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D2A520A1-4459-4DB5-979E-492C784A98C1}"/>
+  <xr:revisionPtr revIDLastSave="103" documentId="11_F25DC773A252ABDACC1048DAA15A48A85ADE58E8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{280A1E25-BA16-40CE-B93F-D631DED76236}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="480" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="480" windowWidth="16440" windowHeight="28440" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -130,24 +130,30 @@
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|14049501234159561198</stp>
-        <tr r="C1" s="2"/>
+        <stp>BDH|14526925194529567840</stp>
+        <tr r="D1" s="2"/>
+      </tp>
+    </main>
+    <main first="bofaddin.rtdserver">
+      <tp t="s">
+        <v>#N/A N/A</v>
+        <stp/>
+        <stp>BDH|9057621605400441360</stp>
+        <tr r="A1" s="2"/>
       </tp>
       <tp t="s">
         <v>#N/A N/A</v>
         <stp/>
-        <stp>BDH|12379947721503079785</stp>
-        <tr r="D1" s="2"/>
-      </tp>
-      <tp t="s">
-        <v>#N/A N/A</v>
-        <stp/>
-        <stp>BDH|15766224238042511682</stp>
-        <tr r="A1" s="2"/>
+        <stp>BDH|2642277049738013257</stp>
+        <tr r="C1" s="2"/>
       </tp>
     </main>
   </volType>
 </volTypes>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -413,7 +419,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1872"/>
+  <dimension ref="A1:C1875"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
@@ -20660,7 +20666,7 @@
       </c>
     </row>
     <row r="1841" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1841">
+      <c r="A1841" s="1">
         <v>45878</v>
       </c>
       <c r="B1841">
@@ -20671,7 +20677,7 @@
       </c>
     </row>
     <row r="1842" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1842">
+      <c r="A1842" s="1">
         <v>45879</v>
       </c>
       <c r="B1842">
@@ -20682,7 +20688,7 @@
       </c>
     </row>
     <row r="1843" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1843">
+      <c r="A1843" s="1">
         <v>45880</v>
       </c>
       <c r="B1843">
@@ -20693,7 +20699,7 @@
       </c>
     </row>
     <row r="1844" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1844">
+      <c r="A1844" s="1">
         <v>45881</v>
       </c>
       <c r="B1844">
@@ -20704,7 +20710,7 @@
       </c>
     </row>
     <row r="1845" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1845">
+      <c r="A1845" s="1">
         <v>45882</v>
       </c>
       <c r="B1845">
@@ -20715,7 +20721,7 @@
       </c>
     </row>
     <row r="1846" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1846">
+      <c r="A1846" s="1">
         <v>45883</v>
       </c>
       <c r="B1846">
@@ -20726,7 +20732,7 @@
       </c>
     </row>
     <row r="1847" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1847">
+      <c r="A1847" s="1">
         <v>45884</v>
       </c>
       <c r="B1847">
@@ -20737,7 +20743,7 @@
       </c>
     </row>
     <row r="1848" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1848">
+      <c r="A1848" s="1">
         <v>45885</v>
       </c>
       <c r="B1848">
@@ -20748,7 +20754,7 @@
       </c>
     </row>
     <row r="1849" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1849">
+      <c r="A1849" s="1">
         <v>45886</v>
       </c>
       <c r="B1849">
@@ -20759,7 +20765,7 @@
       </c>
     </row>
     <row r="1850" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1850">
+      <c r="A1850" s="1">
         <v>45887</v>
       </c>
       <c r="B1850">
@@ -20770,7 +20776,7 @@
       </c>
     </row>
     <row r="1851" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1851">
+      <c r="A1851" s="1">
         <v>45888</v>
       </c>
       <c r="B1851">
@@ -20781,7 +20787,7 @@
       </c>
     </row>
     <row r="1852" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1852">
+      <c r="A1852" s="1">
         <v>45889</v>
       </c>
       <c r="B1852">
@@ -20792,7 +20798,7 @@
       </c>
     </row>
     <row r="1853" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1853">
+      <c r="A1853" s="1">
         <v>45890</v>
       </c>
       <c r="B1853">
@@ -20803,7 +20809,7 @@
       </c>
     </row>
     <row r="1854" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1854">
+      <c r="A1854" s="1">
         <v>45891</v>
       </c>
       <c r="B1854">
@@ -20814,7 +20820,7 @@
       </c>
     </row>
     <row r="1855" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1855">
+      <c r="A1855" s="1">
         <v>45892</v>
       </c>
       <c r="B1855">
@@ -20825,7 +20831,7 @@
       </c>
     </row>
     <row r="1856" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1856">
+      <c r="A1856" s="1">
         <v>45893</v>
       </c>
       <c r="B1856">
@@ -20836,7 +20842,7 @@
       </c>
     </row>
     <row r="1857" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1857">
+      <c r="A1857" s="1">
         <v>45894</v>
       </c>
       <c r="B1857">
@@ -20847,7 +20853,7 @@
       </c>
     </row>
     <row r="1858" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1858">
+      <c r="A1858" s="1">
         <v>45895</v>
       </c>
       <c r="B1858">
@@ -20858,7 +20864,7 @@
       </c>
     </row>
     <row r="1859" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1859">
+      <c r="A1859" s="1">
         <v>45896</v>
       </c>
       <c r="B1859">
@@ -20869,7 +20875,7 @@
       </c>
     </row>
     <row r="1860" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1860">
+      <c r="A1860" s="1">
         <v>45897</v>
       </c>
       <c r="B1860">
@@ -20880,7 +20886,7 @@
       </c>
     </row>
     <row r="1861" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1861">
+      <c r="A1861" s="1">
         <v>45898</v>
       </c>
       <c r="B1861">
@@ -20891,7 +20897,7 @@
       </c>
     </row>
     <row r="1862" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1862">
+      <c r="A1862" s="1">
         <v>45899</v>
       </c>
       <c r="B1862">
@@ -20902,7 +20908,7 @@
       </c>
     </row>
     <row r="1863" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1863">
+      <c r="A1863" s="1">
         <v>45900</v>
       </c>
       <c r="B1863">
@@ -20913,7 +20919,7 @@
       </c>
     </row>
     <row r="1864" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1864">
+      <c r="A1864" s="1">
         <v>45901</v>
       </c>
       <c r="B1864">
@@ -20924,7 +20930,7 @@
       </c>
     </row>
     <row r="1865" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1865">
+      <c r="A1865" s="1">
         <v>45902</v>
       </c>
       <c r="B1865">
@@ -20935,7 +20941,7 @@
       </c>
     </row>
     <row r="1866" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1866">
+      <c r="A1866" s="1">
         <v>45903</v>
       </c>
       <c r="B1866">
@@ -20946,7 +20952,7 @@
       </c>
     </row>
     <row r="1867" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1867">
+      <c r="A1867" s="1">
         <v>45904</v>
       </c>
       <c r="B1867">
@@ -20957,7 +20963,7 @@
       </c>
     </row>
     <row r="1868" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1868">
+      <c r="A1868" s="1">
         <v>45905</v>
       </c>
       <c r="B1868">
@@ -20968,7 +20974,7 @@
       </c>
     </row>
     <row r="1869" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1869">
+      <c r="A1869" s="1">
         <v>45906</v>
       </c>
       <c r="B1869">
@@ -20979,7 +20985,7 @@
       </c>
     </row>
     <row r="1870" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1870">
+      <c r="A1870" s="1">
         <v>45907</v>
       </c>
       <c r="B1870">
@@ -20990,7 +20996,7 @@
       </c>
     </row>
     <row r="1871" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1871">
+      <c r="A1871" s="1">
         <v>45908</v>
       </c>
       <c r="B1871">
@@ -21001,7 +21007,7 @@
       </c>
     </row>
     <row r="1872" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1872">
+      <c r="A1872" s="1">
         <v>45909</v>
       </c>
       <c r="B1872">
@@ -21010,6 +21016,31 @@
       <c r="C1872">
         <v>-2.2865000000000002</v>
       </c>
+    </row>
+    <row r="1873" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1873" s="1">
+        <v>45910</v>
+      </c>
+      <c r="B1873">
+        <v>19.921600000000002</v>
+      </c>
+      <c r="C1873">
+        <v>-2.2214</v>
+      </c>
+    </row>
+    <row r="1874" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1874" s="1">
+        <v>45911</v>
+      </c>
+      <c r="B1874">
+        <v>19.860399999999998</v>
+      </c>
+      <c r="C1874">
+        <v>-2.1964999999999999</v>
+      </c>
+    </row>
+    <row r="1875" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1875" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -21019,25 +21050,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C44AB31A-70CE-4A6E-A84E-7592026AAEFA}">
   <dimension ref="A1:E1873"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="0" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="9.140625" collapsed="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" cm="1">
-        <f t="array" ref="A1:B1871">_xll.BDH("HSTECH Index", "BEST_PE_RATIO", "7/27/2020", "9/9/2025", "Days", "C", "BEST_FPERIOD_OVERRIDE", "1BF")</f>
+        <f t="array" ref="A1:B1873">_xll.BDH("HSTECH Index", "BEST_PE_RATIO", "7/27/2020", "9/11/2025", "Days", "C", "BEST_FPERIOD_OVERRIDE", "1BF")</f>
         <v>44039</v>
       </c>
       <c r="B1">
         <v>31.747399999999999</v>
       </c>
       <c r="C1" cm="1">
-        <f t="array" ref="C1:C1871">_xll.BDH("GCNY10YR Index", "PX_LAST", "7/27/2020", "9/9/2025", "Days", "C", "Dates", "Hide")</f>
+        <f t="array" ref="C1:C1873">_xll.BDH("GCNY10YR Index", "PX_LAST", "7/27/2020", "9/11/2025", "Days", "C", "Dates", "Hide")</f>
         <v>2.8959999999999999</v>
       </c>
       <c r="D1" cm="1">
-        <f t="array" ref="D1:D1871">_xll.BDH("USGG10YR Index", "PX_LAST", "7/27/2020", "9/9/2025", "Days", "C", "Dates", "Hide")</f>
+        <f t="array" ref="D1:D1873">_xll.BDH("USGG10YR Index", "PX_LAST", "7/27/2020", "9/11/2025", "Days", "C", "Dates", "Hide")</f>
         <v>0.61509999999999998</v>
       </c>
       <c r="E1">
@@ -44216,7 +44249,7 @@
         <v>45327</v>
       </c>
       <c r="B1289">
-        <v>12.9008</v>
+        <v>12.900700000000001</v>
       </c>
       <c r="C1289">
         <v>2.4020000000000001</v>
@@ -45368,7 +45401,7 @@
         <v>45391</v>
       </c>
       <c r="B1353">
-        <v>14.510300000000001</v>
+        <v>14.510199999999999</v>
       </c>
       <c r="C1353">
         <v>2.2890000000000001</v>
@@ -45440,7 +45473,7 @@
         <v>45395</v>
       </c>
       <c r="B1357">
-        <v>14.5069</v>
+        <v>14.5068</v>
       </c>
       <c r="C1357">
         <v>2.2839999999999998</v>
@@ -45458,7 +45491,7 @@
         <v>45396</v>
       </c>
       <c r="B1358">
-        <v>14.5036</v>
+        <v>14.503500000000001</v>
       </c>
       <c r="C1358">
         <v>2.2839999999999998</v>
@@ -45476,7 +45509,7 @@
         <v>45397</v>
       </c>
       <c r="B1359">
-        <v>14.382300000000001</v>
+        <v>14.382199999999999</v>
       </c>
       <c r="C1359">
         <v>2.2810000000000001</v>
@@ -45494,7 +45527,7 @@
         <v>45398</v>
       </c>
       <c r="B1360">
-        <v>13.9412</v>
+        <v>13.9411</v>
       </c>
       <c r="C1360">
         <v>2.2719999999999998</v>
@@ -45710,7 +45743,7 @@
         <v>45410</v>
       </c>
       <c r="B1372">
-        <v>15.5145</v>
+        <v>15.5144</v>
       </c>
       <c r="C1372">
         <v>2.306</v>
@@ -45764,7 +45797,7 @@
         <v>45413</v>
       </c>
       <c r="B1375">
-        <v>15.430400000000001</v>
+        <v>15.430300000000001</v>
       </c>
       <c r="C1375">
         <v>2.3140000000000001</v>
@@ -45782,7 +45815,7 @@
         <v>45414</v>
       </c>
       <c r="B1376">
-        <v>16.100300000000001</v>
+        <v>16.100200000000001</v>
       </c>
       <c r="C1376">
         <v>2.3140000000000001</v>
@@ -45836,7 +45869,7 @@
         <v>45417</v>
       </c>
       <c r="B1379">
-        <v>16.5364</v>
+        <v>16.536300000000001</v>
       </c>
       <c r="C1379">
         <v>2.3140000000000001</v>
@@ -45872,7 +45905,7 @@
         <v>45419</v>
       </c>
       <c r="B1381">
-        <v>16.270800000000001</v>
+        <v>16.270700000000001</v>
       </c>
       <c r="C1381">
         <v>2.2890000000000001</v>
@@ -45890,7 +45923,7 @@
         <v>45420</v>
       </c>
       <c r="B1382">
-        <v>16.0609</v>
+        <v>16.0608</v>
       </c>
       <c r="C1382">
         <v>2.298</v>
@@ -45908,7 +45941,7 @@
         <v>45421</v>
       </c>
       <c r="B1383">
-        <v>16.342400000000001</v>
+        <v>16.342300000000002</v>
       </c>
       <c r="C1383">
         <v>2.3159999999999998</v>
@@ -45926,7 +45959,7 @@
         <v>45422</v>
       </c>
       <c r="B1384">
-        <v>16.4194</v>
+        <v>16.4193</v>
       </c>
       <c r="C1384">
         <v>2.3199999999999998</v>
@@ -45962,7 +45995,7 @@
         <v>45424</v>
       </c>
       <c r="B1386">
-        <v>16.394600000000001</v>
+        <v>16.394500000000001</v>
       </c>
       <c r="C1386">
         <v>2.3199999999999998</v>
@@ -45998,7 +46031,7 @@
         <v>45426</v>
       </c>
       <c r="B1388">
-        <v>16.749700000000001</v>
+        <v>16.749600000000001</v>
       </c>
       <c r="C1388">
         <v>2.2919999999999998</v>
@@ -46016,7 +46049,7 @@
         <v>45427</v>
       </c>
       <c r="B1389">
-        <v>16.705400000000001</v>
+        <v>16.705300000000001</v>
       </c>
       <c r="C1389">
         <v>2.3010000000000002</v>
@@ -46034,7 +46067,7 @@
         <v>45428</v>
       </c>
       <c r="B1390">
-        <v>16.7807</v>
+        <v>16.7806</v>
       </c>
       <c r="C1390">
         <v>2.3149999999999999</v>
@@ -46070,7 +46103,7 @@
         <v>45430</v>
       </c>
       <c r="B1392">
-        <v>16.869800000000001</v>
+        <v>16.869700000000002</v>
       </c>
       <c r="C1392">
         <v>2.3170000000000002</v>
@@ -46106,7 +46139,7 @@
         <v>45432</v>
       </c>
       <c r="B1394">
-        <v>16.973099999999999</v>
+        <v>16.972999999999999</v>
       </c>
       <c r="C1394">
         <v>2.3090000000000002</v>
@@ -46124,7 +46157,7 @@
         <v>45433</v>
       </c>
       <c r="B1395">
-        <v>16.353899999999999</v>
+        <v>16.352900000000002</v>
       </c>
       <c r="C1395">
         <v>2.3130000000000002</v>
@@ -46142,7 +46175,7 @@
         <v>45434</v>
       </c>
       <c r="B1396">
-        <v>16.3246</v>
+        <v>16.323599999999999</v>
       </c>
       <c r="C1396">
         <v>2.3119999999999998</v>
@@ -46160,7 +46193,7 @@
         <v>45435</v>
       </c>
       <c r="B1397">
-        <v>15.802199999999999</v>
+        <v>15.8011</v>
       </c>
       <c r="C1397">
         <v>2.306</v>
@@ -46178,7 +46211,7 @@
         <v>45436</v>
       </c>
       <c r="B1398">
-        <v>15.348599999999999</v>
+        <v>15.3476</v>
       </c>
       <c r="C1398">
         <v>2.3140000000000001</v>
@@ -46196,7 +46229,7 @@
         <v>45437</v>
       </c>
       <c r="B1399">
-        <v>15.3323</v>
+        <v>15.331200000000001</v>
       </c>
       <c r="C1399">
         <v>2.3140000000000001</v>
@@ -46214,7 +46247,7 @@
         <v>45438</v>
       </c>
       <c r="B1400">
-        <v>15.3302</v>
+        <v>15.3292</v>
       </c>
       <c r="C1400">
         <v>2.3140000000000001</v>
@@ -46232,7 +46265,7 @@
         <v>45439</v>
       </c>
       <c r="B1401">
-        <v>15.572900000000001</v>
+        <v>15.5716</v>
       </c>
       <c r="C1401">
         <v>2.3130000000000002</v>
@@ -46250,7 +46283,7 @@
         <v>45440</v>
       </c>
       <c r="B1402">
-        <v>15.5121</v>
+        <v>15.5108</v>
       </c>
       <c r="C1402">
         <v>2.2999999999999998</v>
@@ -46268,7 +46301,7 @@
         <v>45441</v>
       </c>
       <c r="B1403">
-        <v>15.124499999999999</v>
+        <v>15.1233</v>
       </c>
       <c r="C1403">
         <v>2.2959999999999998</v>
@@ -46286,7 +46319,7 @@
         <v>45442</v>
       </c>
       <c r="B1404">
-        <v>15.039099999999999</v>
+        <v>15.0379</v>
       </c>
       <c r="C1404">
         <v>2.306</v>
@@ -46304,7 +46337,7 @@
         <v>45443</v>
       </c>
       <c r="B1405">
-        <v>14.8043</v>
+        <v>14.803100000000001</v>
       </c>
       <c r="C1405">
         <v>2.319</v>
@@ -46322,7 +46355,7 @@
         <v>45444</v>
       </c>
       <c r="B1406">
-        <v>14.7927</v>
+        <v>14.791499999999999</v>
       </c>
       <c r="C1406">
         <v>2.319</v>
@@ -46340,7 +46373,7 @@
         <v>45445</v>
       </c>
       <c r="B1407">
-        <v>14.8186</v>
+        <v>14.817399999999999</v>
       </c>
       <c r="C1407">
         <v>2.319</v>
@@ -46358,7 +46391,7 @@
         <v>45446</v>
       </c>
       <c r="B1408">
-        <v>15.1922</v>
+        <v>15.191000000000001</v>
       </c>
       <c r="C1408">
         <v>2.3109999999999999</v>
@@ -46376,7 +46409,7 @@
         <v>45447</v>
       </c>
       <c r="B1409">
-        <v>15.229799999999999</v>
+        <v>15.229699999999999</v>
       </c>
       <c r="C1409">
         <v>2.31</v>
@@ -46412,7 +46445,7 @@
         <v>45449</v>
       </c>
       <c r="B1411">
-        <v>15.346500000000001</v>
+        <v>15.346399999999999</v>
       </c>
       <c r="C1411">
         <v>2.3069999999999999</v>
@@ -46430,7 +46463,7 @@
         <v>45450</v>
       </c>
       <c r="B1412">
-        <v>15.0268</v>
+        <v>15.0267</v>
       </c>
       <c r="C1412">
         <v>2.31</v>
@@ -46520,7 +46553,7 @@
         <v>45455</v>
       </c>
       <c r="B1417">
-        <v>14.788</v>
+        <v>14.7879</v>
       </c>
       <c r="C1417">
         <v>2.306</v>
@@ -46538,7 +46571,7 @@
         <v>45456</v>
       </c>
       <c r="B1418">
-        <v>14.9711</v>
+        <v>14.971</v>
       </c>
       <c r="C1418">
         <v>2.2999999999999998</v>
@@ -46556,7 +46589,7 @@
         <v>45457</v>
       </c>
       <c r="B1419">
-        <v>14.84</v>
+        <v>14.8399</v>
       </c>
       <c r="C1419">
         <v>2.2970000000000002</v>
@@ -46574,7 +46607,7 @@
         <v>45458</v>
       </c>
       <c r="B1420">
-        <v>14.8307</v>
+        <v>14.8306</v>
       </c>
       <c r="C1420">
         <v>2.2970000000000002</v>
@@ -46592,7 +46625,7 @@
         <v>45459</v>
       </c>
       <c r="B1421">
-        <v>14.832100000000001</v>
+        <v>14.832000000000001</v>
       </c>
       <c r="C1421">
         <v>2.2970000000000002</v>
@@ -46628,7 +46661,7 @@
         <v>45461</v>
       </c>
       <c r="B1423">
-        <v>14.7849</v>
+        <v>14.784800000000001</v>
       </c>
       <c r="C1423">
         <v>2.2549999999999999</v>
@@ -46646,7 +46679,7 @@
         <v>45462</v>
       </c>
       <c r="B1424">
-        <v>15.324299999999999</v>
+        <v>15.324199999999999</v>
       </c>
       <c r="C1424">
         <v>2.246</v>
@@ -46664,7 +46697,7 @@
         <v>45463</v>
       </c>
       <c r="B1425">
-        <v>15.0725</v>
+        <v>15.0724</v>
       </c>
       <c r="C1425">
         <v>2.2469999999999999</v>
@@ -46682,7 +46715,7 @@
         <v>45464</v>
       </c>
       <c r="B1426">
-        <v>14.7905</v>
+        <v>14.7904</v>
       </c>
       <c r="C1426">
         <v>2.2599999999999998</v>
@@ -46700,7 +46733,7 @@
         <v>45465</v>
       </c>
       <c r="B1427">
-        <v>14.778700000000001</v>
+        <v>14.778600000000001</v>
       </c>
       <c r="C1427">
         <v>2.2599999999999998</v>
@@ -46736,7 +46769,7 @@
         <v>45467</v>
       </c>
       <c r="B1429">
-        <v>14.682</v>
+        <v>14.681900000000001</v>
       </c>
       <c r="C1429">
         <v>2.2519999999999998</v>
@@ -46754,7 +46787,7 @@
         <v>45468</v>
       </c>
       <c r="B1430">
-        <v>14.591900000000001</v>
+        <v>14.591799999999999</v>
       </c>
       <c r="C1430">
         <v>2.2330000000000001</v>
@@ -46772,7 +46805,7 @@
         <v>45469</v>
       </c>
       <c r="B1431">
-        <v>14.7189</v>
+        <v>14.7188</v>
       </c>
       <c r="C1431">
         <v>2.226</v>
@@ -46808,7 +46841,7 @@
         <v>45471</v>
       </c>
       <c r="B1433">
-        <v>14.143800000000001</v>
+        <v>14.143700000000001</v>
       </c>
       <c r="C1433">
         <v>2.21</v>
@@ -46826,7 +46859,7 @@
         <v>45472</v>
       </c>
       <c r="B1434">
-        <v>14.134600000000001</v>
+        <v>14.134499999999999</v>
       </c>
       <c r="C1434">
         <v>2.21</v>
@@ -46844,7 +46877,7 @@
         <v>45473</v>
       </c>
       <c r="B1435">
-        <v>14.1249</v>
+        <v>14.1248</v>
       </c>
       <c r="C1435">
         <v>2.21</v>
@@ -46862,7 +46895,7 @@
         <v>45474</v>
       </c>
       <c r="B1436">
-        <v>14.1153</v>
+        <v>14.1152</v>
       </c>
       <c r="C1436">
         <v>2.2530000000000001</v>
@@ -46880,7 +46913,7 @@
         <v>45475</v>
       </c>
       <c r="B1437">
-        <v>14.0519</v>
+        <v>14.0518</v>
       </c>
       <c r="C1437">
         <v>2.2400000000000002</v>
@@ -46898,7 +46931,7 @@
         <v>45476</v>
       </c>
       <c r="B1438">
-        <v>14.391500000000001</v>
+        <v>14.391400000000001</v>
       </c>
       <c r="C1438">
         <v>2.2429999999999999</v>
@@ -46916,7 +46949,7 @@
         <v>45477</v>
       </c>
       <c r="B1439">
-        <v>14.476800000000001</v>
+        <v>14.476699999999999</v>
       </c>
       <c r="C1439">
         <v>2.2490000000000001</v>
@@ -46934,7 +46967,7 @@
         <v>45478</v>
       </c>
       <c r="B1440">
-        <v>14.2652</v>
+        <v>14.2651</v>
       </c>
       <c r="C1440">
         <v>2.2730000000000001</v>
@@ -46988,7 +47021,7 @@
         <v>45481</v>
       </c>
       <c r="B1443">
-        <v>14.1189</v>
+        <v>14.1188</v>
       </c>
       <c r="C1443">
         <v>2.29</v>
@@ -47042,7 +47075,7 @@
         <v>45484</v>
       </c>
       <c r="B1446">
-        <v>14.566000000000001</v>
+        <v>14.565899999999999</v>
       </c>
       <c r="C1446">
         <v>2.2639999999999998</v>
@@ -47078,7 +47111,7 @@
         <v>45486</v>
       </c>
       <c r="B1448">
-        <v>14.856299999999999</v>
+        <v>14.856199999999999</v>
       </c>
       <c r="C1448">
         <v>2.2589999999999999</v>
@@ -47114,7 +47147,7 @@
         <v>45488</v>
       </c>
       <c r="B1450">
-        <v>14.4095</v>
+        <v>14.4094</v>
       </c>
       <c r="C1450">
         <v>2.25</v>
@@ -48248,7 +48281,7 @@
         <v>45551</v>
       </c>
       <c r="B1513">
-        <v>12.6442</v>
+        <v>12.6439</v>
       </c>
       <c r="C1513">
         <v>2.073</v>
@@ -48266,7 +48299,7 @@
         <v>45552</v>
       </c>
       <c r="B1514">
-        <v>12.7761</v>
+        <v>12.7758</v>
       </c>
       <c r="C1514">
         <v>2.073</v>
@@ -48284,7 +48317,7 @@
         <v>45553</v>
       </c>
       <c r="B1515">
-        <v>12.760899999999999</v>
+        <v>12.7606</v>
       </c>
       <c r="C1515">
         <v>2.04</v>
@@ -48302,7 +48335,7 @@
         <v>45554</v>
       </c>
       <c r="B1516">
-        <v>13.139200000000001</v>
+        <v>13.1389</v>
       </c>
       <c r="C1516">
         <v>2.0449999999999999</v>
@@ -48320,7 +48353,7 @@
         <v>45555</v>
       </c>
       <c r="B1517">
-        <v>13.2613</v>
+        <v>13.260999999999999</v>
       </c>
       <c r="C1517">
         <v>2.0409999999999999</v>
@@ -48338,7 +48371,7 @@
         <v>45556</v>
       </c>
       <c r="B1518">
-        <v>13.245699999999999</v>
+        <v>13.2454</v>
       </c>
       <c r="C1518">
         <v>2.0409999999999999</v>
@@ -48356,7 +48389,7 @@
         <v>45557</v>
       </c>
       <c r="B1519">
-        <v>13.240500000000001</v>
+        <v>13.2402</v>
       </c>
       <c r="C1519">
         <v>2.0409999999999999</v>
@@ -48374,7 +48407,7 @@
         <v>45558</v>
       </c>
       <c r="B1520">
-        <v>13.223000000000001</v>
+        <v>13.2226</v>
       </c>
       <c r="C1520">
         <v>2.0369999999999999</v>
@@ -48392,7 +48425,7 @@
         <v>45559</v>
       </c>
       <c r="B1521">
-        <v>13.9655</v>
+        <v>13.965199999999999</v>
       </c>
       <c r="C1521">
         <v>2.0630000000000002</v>
@@ -48410,7 +48443,7 @@
         <v>45560</v>
       </c>
       <c r="B1522">
-        <v>13.9855</v>
+        <v>13.985099999999999</v>
       </c>
       <c r="C1522">
         <v>2.0379999999999998</v>
@@ -48428,7 +48461,7 @@
         <v>45561</v>
       </c>
       <c r="B1523">
-        <v>14.976800000000001</v>
+        <v>14.9765</v>
       </c>
       <c r="C1523">
         <v>2.081</v>
@@ -48446,7 +48479,7 @@
         <v>45562</v>
       </c>
       <c r="B1524">
-        <v>15.831200000000001</v>
+        <v>15.8308</v>
       </c>
       <c r="C1524">
         <v>2.1829999999999998</v>
@@ -48464,7 +48497,7 @@
         <v>45563</v>
       </c>
       <c r="B1525">
-        <v>15.819699999999999</v>
+        <v>15.8193</v>
       </c>
       <c r="C1525">
         <v>2.1829999999999998</v>
@@ -48482,7 +48515,7 @@
         <v>45564</v>
       </c>
       <c r="B1526">
-        <v>15.805899999999999</v>
+        <v>15.8055</v>
       </c>
       <c r="C1526">
         <v>2.1829999999999998</v>
@@ -48500,7 +48533,7 @@
         <v>45565</v>
       </c>
       <c r="B1527">
-        <v>16.864799999999999</v>
+        <v>16.8643</v>
       </c>
       <c r="C1527">
         <v>2.21</v>
@@ -48518,7 +48551,7 @@
         <v>45566</v>
       </c>
       <c r="B1528">
-        <v>16.850999999999999</v>
+        <v>16.8505</v>
       </c>
       <c r="C1528">
         <v>2.21</v>
@@ -48536,7 +48569,7 @@
         <v>45567</v>
       </c>
       <c r="B1529">
-        <v>18.275700000000001</v>
+        <v>18.275200000000002</v>
       </c>
       <c r="C1529">
         <v>2.21</v>
@@ -48554,7 +48587,7 @@
         <v>45568</v>
       </c>
       <c r="B1530">
-        <v>17.6296</v>
+        <v>17.629200000000001</v>
       </c>
       <c r="C1530">
         <v>2.21</v>
@@ -48572,7 +48605,7 @@
         <v>45569</v>
       </c>
       <c r="B1531">
-        <v>18.499199999999998</v>
+        <v>18.498699999999999</v>
       </c>
       <c r="C1531">
         <v>2.21</v>
@@ -48590,7 +48623,7 @@
         <v>45570</v>
       </c>
       <c r="B1532">
-        <v>18.488099999999999</v>
+        <v>18.4876</v>
       </c>
       <c r="C1532">
         <v>2.21</v>
@@ -48608,7 +48641,7 @@
         <v>45571</v>
       </c>
       <c r="B1533">
-        <v>18.489599999999999</v>
+        <v>18.489100000000001</v>
       </c>
       <c r="C1533">
         <v>2.21</v>
@@ -48626,7 +48659,7 @@
         <v>45572</v>
       </c>
       <c r="B1534">
-        <v>19.026499999999999</v>
+        <v>19.026</v>
       </c>
       <c r="C1534">
         <v>2.21</v>
@@ -48644,7 +48677,7 @@
         <v>45573</v>
       </c>
       <c r="B1535">
-        <v>16.636199999999999</v>
+        <v>16.6357</v>
       </c>
       <c r="C1535">
         <v>2.2090000000000001</v>
@@ -48662,7 +48695,7 @@
         <v>45574</v>
       </c>
       <c r="B1536">
-        <v>16.477</v>
+        <v>16.476500000000001</v>
       </c>
       <c r="C1536">
         <v>2.1859999999999999</v>
@@ -48680,7 +48713,7 @@
         <v>45575</v>
       </c>
       <c r="B1537">
-        <v>16.812899999999999</v>
+        <v>16.8125</v>
       </c>
       <c r="C1537">
         <v>2.157</v>
@@ -48698,7 +48731,7 @@
         <v>45576</v>
       </c>
       <c r="B1538">
-        <v>16.791699999999999</v>
+        <v>16.7913</v>
       </c>
       <c r="C1538">
         <v>2.1469999999999998</v>
@@ -48716,7 +48749,7 @@
         <v>45577</v>
       </c>
       <c r="B1539">
-        <v>16.791799999999999</v>
+        <v>16.7913</v>
       </c>
       <c r="C1539">
         <v>2.1469999999999998</v>
@@ -48734,7 +48767,7 @@
         <v>45578</v>
       </c>
       <c r="B1540">
-        <v>16.787099999999999</v>
+        <v>16.7867</v>
       </c>
       <c r="C1540">
         <v>2.1469999999999998</v>
@@ -48752,7 +48785,7 @@
         <v>45579</v>
       </c>
       <c r="B1541">
-        <v>16.567299999999999</v>
+        <v>16.566800000000001</v>
       </c>
       <c r="C1541">
         <v>2.149</v>
@@ -48770,7 +48803,7 @@
         <v>45580</v>
       </c>
       <c r="B1542">
-        <v>15.832700000000001</v>
+        <v>15.8323</v>
       </c>
       <c r="C1542">
         <v>2.1459999999999999</v>
@@ -48788,7 +48821,7 @@
         <v>45581</v>
       </c>
       <c r="B1543">
-        <v>15.6296</v>
+        <v>15.629200000000001</v>
       </c>
       <c r="C1543">
         <v>2.1360000000000001</v>
@@ -48806,7 +48839,7 @@
         <v>45582</v>
       </c>
       <c r="B1544">
-        <v>15.4376</v>
+        <v>15.437200000000001</v>
       </c>
       <c r="C1544">
         <v>2.1179999999999999</v>
@@ -48824,7 +48857,7 @@
         <v>45583</v>
       </c>
       <c r="B1545">
-        <v>16.300999999999998</v>
+        <v>16.300599999999999</v>
       </c>
       <c r="C1545">
         <v>2.1230000000000002</v>
@@ -48842,7 +48875,7 @@
         <v>45584</v>
       </c>
       <c r="B1546">
-        <v>16.2913</v>
+        <v>16.290900000000001</v>
       </c>
       <c r="C1546">
         <v>2.1230000000000002</v>
@@ -48860,7 +48893,7 @@
         <v>45585</v>
       </c>
       <c r="B1547">
-        <v>16.287400000000002</v>
+        <v>16.286899999999999</v>
       </c>
       <c r="C1547">
         <v>2.1230000000000002</v>
@@ -48878,7 +48911,7 @@
         <v>45586</v>
       </c>
       <c r="B1548">
-        <v>15.9076</v>
+        <v>15.9072</v>
       </c>
       <c r="C1548">
         <v>2.1190000000000002</v>
@@ -48896,7 +48929,7 @@
         <v>45587</v>
       </c>
       <c r="B1549">
-        <v>15.996</v>
+        <v>15.9956</v>
       </c>
       <c r="C1549">
         <v>2.141</v>
@@ -48914,7 +48947,7 @@
         <v>45588</v>
       </c>
       <c r="B1550">
-        <v>16.302499999999998</v>
+        <v>16.302099999999999</v>
       </c>
       <c r="C1550">
         <v>2.1579999999999999</v>
@@ -48932,7 +48965,7 @@
         <v>45589</v>
       </c>
       <c r="B1551">
-        <v>15.8653</v>
+        <v>15.8649</v>
       </c>
       <c r="C1551">
         <v>2.161</v>
@@ -48950,7 +48983,7 @@
         <v>45590</v>
       </c>
       <c r="B1552">
-        <v>16.0535</v>
+        <v>16.053100000000001</v>
       </c>
       <c r="C1552">
         <v>2.1579999999999999</v>
@@ -48968,7 +49001,7 @@
         <v>45591</v>
       </c>
       <c r="B1553">
-        <v>16.044</v>
+        <v>16.043500000000002</v>
       </c>
       <c r="C1553">
         <v>2.1579999999999999</v>
@@ -48986,7 +49019,7 @@
         <v>45592</v>
       </c>
       <c r="B1554">
-        <v>16.042300000000001</v>
+        <v>16.041799999999999</v>
       </c>
       <c r="C1554">
         <v>2.1579999999999999</v>
@@ -49004,7 +49037,7 @@
         <v>45593</v>
       </c>
       <c r="B1555">
-        <v>16.1614</v>
+        <v>16.160900000000002</v>
       </c>
       <c r="C1555">
         <v>2.1619999999999999</v>
@@ -49022,7 +49055,7 @@
         <v>45594</v>
       </c>
       <c r="B1556">
-        <v>16.337599999999998</v>
+        <v>16.337199999999999</v>
       </c>
       <c r="C1556">
         <v>2.1589999999999998</v>
@@ -51902,7 +51935,7 @@
         <v>45754</v>
       </c>
       <c r="B1716">
-        <v>13.9955</v>
+        <v>13.991300000000001</v>
       </c>
       <c r="C1716">
         <v>1.64</v>
@@ -51920,7 +51953,7 @@
         <v>45755</v>
       </c>
       <c r="B1717">
-        <v>14.535600000000001</v>
+        <v>14.5312</v>
       </c>
       <c r="C1717">
         <v>1.6659999999999999</v>
@@ -51938,7 +51971,7 @@
         <v>45756</v>
       </c>
       <c r="B1718">
-        <v>14.9526</v>
+        <v>14.948</v>
       </c>
       <c r="C1718">
         <v>1.6519999999999999</v>
@@ -51956,7 +51989,7 @@
         <v>45757</v>
       </c>
       <c r="B1719">
-        <v>15.3231</v>
+        <v>15.3186</v>
       </c>
       <c r="C1719">
         <v>1.6519999999999999</v>
@@ -51974,7 +52007,7 @@
         <v>45758</v>
       </c>
       <c r="B1720">
-        <v>15.5661</v>
+        <v>15.561500000000001</v>
       </c>
       <c r="C1720">
         <v>1.6579999999999999</v>
@@ -51992,7 +52025,7 @@
         <v>45759</v>
       </c>
       <c r="B1721">
-        <v>15.5525</v>
+        <v>15.5479</v>
       </c>
       <c r="C1721">
         <v>1.6579999999999999</v>
@@ -52010,7 +52043,7 @@
         <v>45760</v>
       </c>
       <c r="B1722">
-        <v>15.5326</v>
+        <v>15.528</v>
       </c>
       <c r="C1722">
         <v>1.6579999999999999</v>
@@ -52028,7 +52061,7 @@
         <v>45761</v>
       </c>
       <c r="B1723">
-        <v>15.9122</v>
+        <v>15.905900000000001</v>
       </c>
       <c r="C1723">
         <v>1.6639999999999999</v>
@@ -52046,7 +52079,7 @@
         <v>45762</v>
       </c>
       <c r="B1724">
-        <v>15.801299999999999</v>
+        <v>15.7949</v>
       </c>
       <c r="C1724">
         <v>1.659</v>
@@ -52064,7 +52097,7 @@
         <v>45763</v>
       </c>
       <c r="B1725">
-        <v>15.1769</v>
+        <v>15.1709</v>
       </c>
       <c r="C1725">
         <v>1.6459999999999999</v>
@@ -52082,7 +52115,7 @@
         <v>45764</v>
       </c>
       <c r="B1726">
-        <v>15.4216</v>
+        <v>15.4155</v>
       </c>
       <c r="C1726">
         <v>1.6539999999999999</v>
@@ -52100,7 +52133,7 @@
         <v>45765</v>
       </c>
       <c r="B1727">
-        <v>15.4061</v>
+        <v>15.4001</v>
       </c>
       <c r="C1727">
         <v>1.65</v>
@@ -52118,7 +52151,7 @@
         <v>45766</v>
       </c>
       <c r="B1728">
-        <v>15.3986</v>
+        <v>15.3926</v>
       </c>
       <c r="C1728">
         <v>1.65</v>
@@ -52136,7 +52169,7 @@
         <v>45767</v>
       </c>
       <c r="B1729">
-        <v>15.385300000000001</v>
+        <v>15.379200000000001</v>
       </c>
       <c r="C1729">
         <v>1.65</v>
@@ -52154,7 +52187,7 @@
         <v>45768</v>
       </c>
       <c r="B1730">
-        <v>15.382999999999999</v>
+        <v>15.377000000000001</v>
       </c>
       <c r="C1730">
         <v>1.6639999999999999</v>
@@ -52172,7 +52205,7 @@
         <v>45769</v>
       </c>
       <c r="B1731">
-        <v>15.437799999999999</v>
+        <v>15.431900000000001</v>
       </c>
       <c r="C1731">
         <v>1.653</v>
@@ -52190,7 +52223,7 @@
         <v>45770</v>
       </c>
       <c r="B1732">
-        <v>15.8727</v>
+        <v>15.8666</v>
       </c>
       <c r="C1732">
         <v>1.6619999999999999</v>
@@ -52208,7 +52241,7 @@
         <v>45771</v>
       </c>
       <c r="B1733">
-        <v>15.621600000000001</v>
+        <v>15.615600000000001</v>
       </c>
       <c r="C1733">
         <v>1.6619999999999999</v>
@@ -52226,7 +52259,7 @@
         <v>45772</v>
       </c>
       <c r="B1734">
-        <v>15.635300000000001</v>
+        <v>15.6294</v>
       </c>
       <c r="C1734">
         <v>1.661</v>
@@ -52244,7 +52277,7 @@
         <v>45773</v>
       </c>
       <c r="B1735">
-        <v>15.622999999999999</v>
+        <v>15.617100000000001</v>
       </c>
       <c r="C1735">
         <v>1.661</v>
@@ -52262,7 +52295,7 @@
         <v>45774</v>
       </c>
       <c r="B1736">
-        <v>15.628299999999999</v>
+        <v>15.6226</v>
       </c>
       <c r="C1736">
         <v>1.661</v>
@@ -52280,7 +52313,7 @@
         <v>45775</v>
       </c>
       <c r="B1737">
-        <v>15.6562</v>
+        <v>15.650600000000001</v>
       </c>
       <c r="C1737">
         <v>1.647</v>
@@ -52298,7 +52331,7 @@
         <v>45776</v>
       </c>
       <c r="B1738">
-        <v>15.715299999999999</v>
+        <v>15.7097</v>
       </c>
       <c r="C1738">
         <v>1.6319999999999999</v>
@@ -52316,7 +52349,7 @@
         <v>45777</v>
       </c>
       <c r="B1739">
-        <v>15.9177</v>
+        <v>15.9107</v>
       </c>
       <c r="C1739">
         <v>1.6279999999999999</v>
@@ -52334,7 +52367,7 @@
         <v>45778</v>
       </c>
       <c r="B1740">
-        <v>15.908300000000001</v>
+        <v>15.902799999999999</v>
       </c>
       <c r="C1740">
         <v>1.6279999999999999</v>
@@ -52352,7 +52385,7 @@
         <v>45779</v>
       </c>
       <c r="B1741">
-        <v>16.380500000000001</v>
+        <v>16.3749</v>
       </c>
       <c r="C1741">
         <v>1.6279999999999999</v>
@@ -52370,7 +52403,7 @@
         <v>45780</v>
       </c>
       <c r="B1742">
-        <v>16.370899999999999</v>
+        <v>16.365300000000001</v>
       </c>
       <c r="C1742">
         <v>1.6279999999999999</v>
@@ -52388,7 +52421,7 @@
         <v>45781</v>
       </c>
       <c r="B1743">
-        <v>16.3673</v>
+        <v>16.361699999999999</v>
       </c>
       <c r="C1743">
         <v>1.6279999999999999</v>
@@ -52406,7 +52439,7 @@
         <v>45782</v>
       </c>
       <c r="B1744">
-        <v>16.342099999999999</v>
+        <v>16.336500000000001</v>
       </c>
       <c r="C1744">
         <v>1.6279999999999999</v>
@@ -52424,7 +52457,7 @@
         <v>45783</v>
       </c>
       <c r="B1745">
-        <v>16.258800000000001</v>
+        <v>16.253299999999999</v>
       </c>
       <c r="C1745">
         <v>1.627</v>
@@ -52442,7 +52475,7 @@
         <v>45784</v>
       </c>
       <c r="B1746">
-        <v>16.126000000000001</v>
+        <v>16.120799999999999</v>
       </c>
       <c r="C1746">
         <v>1.64</v>
@@ -52460,7 +52493,7 @@
         <v>45785</v>
       </c>
       <c r="B1747">
-        <v>16.1921</v>
+        <v>16.186800000000002</v>
       </c>
       <c r="C1747">
         <v>1.629</v>
@@ -52478,7 +52511,7 @@
         <v>45786</v>
       </c>
       <c r="B1748">
-        <v>16.032800000000002</v>
+        <v>16.0276</v>
       </c>
       <c r="C1748">
         <v>1.635</v>
@@ -52496,7 +52529,7 @@
         <v>45787</v>
       </c>
       <c r="B1749">
-        <v>16.0275</v>
+        <v>16.022200000000002</v>
       </c>
       <c r="C1749">
         <v>1.635</v>
@@ -52514,7 +52547,7 @@
         <v>45788</v>
       </c>
       <c r="B1750">
-        <v>16.022600000000001</v>
+        <v>16.017399999999999</v>
       </c>
       <c r="C1750">
         <v>1.635</v>
@@ -52532,7 +52565,7 @@
         <v>45789</v>
       </c>
       <c r="B1751">
-        <v>16.748000000000001</v>
+        <v>16.7425</v>
       </c>
       <c r="C1751">
         <v>1.681</v>
@@ -52550,7 +52583,7 @@
         <v>45790</v>
       </c>
       <c r="B1752">
-        <v>16.2209</v>
+        <v>16.2164</v>
       </c>
       <c r="C1752">
         <v>1.661</v>
@@ -52568,7 +52601,7 @@
         <v>45791</v>
       </c>
       <c r="B1753">
-        <v>16.588799999999999</v>
+        <v>16.5854</v>
       </c>
       <c r="C1753">
         <v>1.671</v>
@@ -52586,7 +52619,7 @@
         <v>45792</v>
       </c>
       <c r="B1754">
-        <v>16.4177</v>
+        <v>16.4147</v>
       </c>
       <c r="C1754">
         <v>1.6759999999999999</v>
@@ -52802,7 +52835,7 @@
         <v>45804</v>
       </c>
       <c r="B1766">
-        <v>16.105599999999999</v>
+        <v>16.107199999999999</v>
       </c>
       <c r="C1766">
         <v>1.7010000000000001</v>
@@ -52820,7 +52853,7 @@
         <v>45805</v>
       </c>
       <c r="B1767">
-        <v>16.0794</v>
+        <v>16.0809</v>
       </c>
       <c r="C1767">
         <v>1.7090000000000001</v>
@@ -52838,7 +52871,7 @@
         <v>45806</v>
       </c>
       <c r="B1768">
-        <v>16.486599999999999</v>
+        <v>16.488099999999999</v>
       </c>
       <c r="C1768">
         <v>1.718</v>
@@ -52856,7 +52889,7 @@
         <v>45807</v>
       </c>
       <c r="B1769">
-        <v>16.109000000000002</v>
+        <v>16.110499999999998</v>
       </c>
       <c r="C1769">
         <v>1.706</v>
@@ -52874,7 +52907,7 @@
         <v>45808</v>
       </c>
       <c r="B1770">
-        <v>16.099</v>
+        <v>16.1005</v>
       </c>
       <c r="C1770">
         <v>1.706</v>
@@ -52892,7 +52925,7 @@
         <v>45809</v>
       </c>
       <c r="B1771">
-        <v>16.087800000000001</v>
+        <v>16.089300000000001</v>
       </c>
       <c r="C1771">
         <v>1.706</v>
@@ -52910,7 +52943,7 @@
         <v>45810</v>
       </c>
       <c r="B1772">
-        <v>16.0091</v>
+        <v>16.0106</v>
       </c>
       <c r="C1772">
         <v>1.706</v>
@@ -52928,7 +52961,7 @@
         <v>45811</v>
       </c>
       <c r="B1773">
-        <v>16.150500000000001</v>
+        <v>16.151900000000001</v>
       </c>
       <c r="C1773">
         <v>1.7070000000000001</v>
@@ -52946,7 +52979,7 @@
         <v>45812</v>
       </c>
       <c r="B1774">
-        <v>16.213699999999999</v>
+        <v>16.215499999999999</v>
       </c>
       <c r="C1774">
         <v>1.704</v>
@@ -52964,7 +52997,7 @@
         <v>45813</v>
       </c>
       <c r="B1775">
-        <v>16.5229</v>
+        <v>16.524699999999999</v>
       </c>
       <c r="C1775">
         <v>1.7030000000000001</v>
@@ -52982,7 +53015,7 @@
         <v>45814</v>
       </c>
       <c r="B1776">
-        <v>16.4419</v>
+        <v>16.4438</v>
       </c>
       <c r="C1776">
         <v>1.6930000000000001</v>
@@ -53000,7 +53033,7 @@
         <v>45815</v>
       </c>
       <c r="B1777">
-        <v>16.4316</v>
+        <v>16.433399999999999</v>
       </c>
       <c r="C1777">
         <v>1.6930000000000001</v>
@@ -53018,7 +53051,7 @@
         <v>45816</v>
       </c>
       <c r="B1778">
-        <v>16.423300000000001</v>
+        <v>16.4251</v>
       </c>
       <c r="C1778">
         <v>1.6930000000000001</v>
@@ -53036,7 +53069,7 @@
         <v>45817</v>
       </c>
       <c r="B1779">
-        <v>16.145299999999999</v>
+        <v>16.146799999999999</v>
       </c>
       <c r="C1779">
         <v>1.6919999999999999</v>
@@ -53054,7 +53087,7 @@
         <v>45818</v>
       </c>
       <c r="B1780">
-        <v>15.3522</v>
+        <v>15.3535</v>
       </c>
       <c r="C1780">
         <v>1.694</v>
@@ -53072,7 +53105,7 @@
         <v>45819</v>
       </c>
       <c r="B1781">
-        <v>15.5124</v>
+        <v>15.5137</v>
       </c>
       <c r="C1781">
         <v>1.6859999999999999</v>
@@ -53090,7 +53123,7 @@
         <v>45820</v>
       </c>
       <c r="B1782">
-        <v>15.1098</v>
+        <v>15.1111</v>
       </c>
       <c r="C1782">
         <v>1.7030000000000001</v>
@@ -53108,7 +53141,7 @@
         <v>45821</v>
       </c>
       <c r="B1783">
-        <v>14.8477</v>
+        <v>14.849</v>
       </c>
       <c r="C1783">
         <v>1.702</v>
@@ -53126,7 +53159,7 @@
         <v>45822</v>
       </c>
       <c r="B1784">
-        <v>14.845000000000001</v>
+        <v>14.846299999999999</v>
       </c>
       <c r="C1784">
         <v>1.702</v>
@@ -53144,7 +53177,7 @@
         <v>45823</v>
       </c>
       <c r="B1785">
-        <v>14.837899999999999</v>
+        <v>14.8392</v>
       </c>
       <c r="C1785">
         <v>1.702</v>
@@ -53162,7 +53195,7 @@
         <v>45824</v>
       </c>
       <c r="B1786">
-        <v>15.027200000000001</v>
+        <v>15.028600000000001</v>
       </c>
       <c r="C1786">
         <v>1.6990000000000001</v>
@@ -53180,7 +53213,7 @@
         <v>45825</v>
       </c>
       <c r="B1787">
-        <v>15.002000000000001</v>
+        <v>15.003299999999999</v>
       </c>
       <c r="C1787">
         <v>1.694</v>
@@ -53198,7 +53231,7 @@
         <v>45826</v>
       </c>
       <c r="B1788">
-        <v>14.7944</v>
+        <v>14.7956</v>
       </c>
       <c r="C1788">
         <v>1.639</v>
@@ -53216,7 +53249,7 @@
         <v>45827</v>
       </c>
       <c r="B1789">
-        <v>14.428100000000001</v>
+        <v>14.4292</v>
       </c>
       <c r="C1789">
         <v>1.6419999999999999</v>
@@ -53234,7 +53267,7 @@
         <v>45828</v>
       </c>
       <c r="B1790">
-        <v>14.539899999999999</v>
+        <v>14.541</v>
       </c>
       <c r="C1790">
         <v>1.639</v>
@@ -53252,7 +53285,7 @@
         <v>45829</v>
       </c>
       <c r="B1791">
-        <v>14.531700000000001</v>
+        <v>14.5328</v>
       </c>
       <c r="C1791">
         <v>1.639</v>
@@ -53270,7 +53303,7 @@
         <v>45830</v>
       </c>
       <c r="B1792">
-        <v>14.5204</v>
+        <v>14.5215</v>
       </c>
       <c r="C1792">
         <v>1.639</v>
@@ -53288,7 +53321,7 @@
         <v>45831</v>
       </c>
       <c r="B1793">
-        <v>14.646000000000001</v>
+        <v>14.647500000000001</v>
       </c>
       <c r="C1793">
         <v>1.6419999999999999</v>
@@ -53306,7 +53339,7 @@
         <v>45832</v>
       </c>
       <c r="B1794">
-        <v>14.9621</v>
+        <v>14.9636</v>
       </c>
       <c r="C1794">
         <v>1.649</v>
@@ -53324,7 +53357,7 @@
         <v>45833</v>
       </c>
       <c r="B1795">
-        <v>15.130100000000001</v>
+        <v>15.1317</v>
       </c>
       <c r="C1795">
         <v>1.655</v>
@@ -53342,7 +53375,7 @@
         <v>45834</v>
       </c>
       <c r="B1796">
-        <v>15.0528</v>
+        <v>15.0543</v>
       </c>
       <c r="C1796">
         <v>1.647</v>
@@ -53360,7 +53393,7 @@
         <v>45835</v>
       </c>
       <c r="B1797">
-        <v>15.0342</v>
+        <v>15.0358</v>
       </c>
       <c r="C1797">
         <v>1.6479999999999999</v>
@@ -53378,7 +53411,7 @@
         <v>45836</v>
       </c>
       <c r="B1798">
-        <v>15.0258</v>
+        <v>15.0273</v>
       </c>
       <c r="C1798">
         <v>1.6479999999999999</v>
@@ -53396,7 +53429,7 @@
         <v>45837</v>
       </c>
       <c r="B1799">
-        <v>15.0296</v>
+        <v>15.0312</v>
       </c>
       <c r="C1799">
         <v>1.6479999999999999</v>
@@ -53414,7 +53447,7 @@
         <v>45838</v>
       </c>
       <c r="B1800">
-        <v>14.896599999999999</v>
+        <v>14.898099999999999</v>
       </c>
       <c r="C1800">
         <v>1.65</v>
@@ -53432,7 +53465,7 @@
         <v>45839</v>
       </c>
       <c r="B1801">
-        <v>14.8919</v>
+        <v>14.8935</v>
       </c>
       <c r="C1801">
         <v>1.647</v>
@@ -53450,7 +53483,7 @@
         <v>45840</v>
       </c>
       <c r="B1802">
-        <v>14.7935</v>
+        <v>14.795</v>
       </c>
       <c r="C1802">
         <v>1.643</v>
@@ -53468,7 +53501,7 @@
         <v>45841</v>
       </c>
       <c r="B1803">
-        <v>14.7014</v>
+        <v>14.702999999999999</v>
       </c>
       <c r="C1803">
         <v>1.643</v>
@@ -53486,7 +53519,7 @@
         <v>45842</v>
       </c>
       <c r="B1804">
-        <v>14.6342</v>
+        <v>14.6357</v>
       </c>
       <c r="C1804">
         <v>1.645</v>
@@ -53504,7 +53537,7 @@
         <v>45843</v>
       </c>
       <c r="B1805">
-        <v>14.625999999999999</v>
+        <v>14.6275</v>
       </c>
       <c r="C1805">
         <v>1.645</v>
@@ -53522,7 +53555,7 @@
         <v>45844</v>
       </c>
       <c r="B1806">
-        <v>14.617599999999999</v>
+        <v>14.6191</v>
       </c>
       <c r="C1806">
         <v>1.645</v>
@@ -53540,7 +53573,7 @@
         <v>45845</v>
       </c>
       <c r="B1807">
-        <v>14.6731</v>
+        <v>14.6746</v>
       </c>
       <c r="C1807">
         <v>1.6439999999999999</v>
@@ -53558,7 +53591,7 @@
         <v>45846</v>
       </c>
       <c r="B1808">
-        <v>14.9534</v>
+        <v>14.955</v>
       </c>
       <c r="C1808">
         <v>1.6479999999999999</v>
@@ -53576,7 +53609,7 @@
         <v>45847</v>
       </c>
       <c r="B1809">
-        <v>14.7149</v>
+        <v>14.7165</v>
       </c>
       <c r="C1809">
         <v>1.6479999999999999</v>
@@ -53594,7 +53627,7 @@
         <v>45848</v>
       </c>
       <c r="B1810">
-        <v>14.8795</v>
+        <v>14.8811</v>
       </c>
       <c r="C1810">
         <v>1.66</v>
@@ -53612,7 +53645,7 @@
         <v>45849</v>
       </c>
       <c r="B1811">
-        <v>15.101699999999999</v>
+        <v>15.1035</v>
       </c>
       <c r="C1811">
         <v>1.6679999999999999</v>
@@ -53630,7 +53663,7 @@
         <v>45850</v>
       </c>
       <c r="B1812">
-        <v>15.110799999999999</v>
+        <v>15.1126</v>
       </c>
       <c r="C1812">
         <v>1.6679999999999999</v>
@@ -53648,7 +53681,7 @@
         <v>45851</v>
       </c>
       <c r="B1813">
-        <v>15.1188</v>
+        <v>15.1206</v>
       </c>
       <c r="C1813">
         <v>1.6679999999999999</v>
@@ -53666,7 +53699,7 @@
         <v>45852</v>
       </c>
       <c r="B1814">
-        <v>15.274900000000001</v>
+        <v>15.2767</v>
       </c>
       <c r="C1814">
         <v>1.6719999999999999</v>
@@ -53684,7 +53717,7 @@
         <v>45853</v>
       </c>
       <c r="B1815">
-        <v>15.766</v>
+        <v>15.767799999999999</v>
       </c>
       <c r="C1815">
         <v>1.659</v>
@@ -53702,7 +53735,7 @@
         <v>45854</v>
       </c>
       <c r="B1816">
-        <v>15.7325</v>
+        <v>15.734400000000001</v>
       </c>
       <c r="C1816">
         <v>1.6619999999999999</v>
@@ -53720,7 +53753,7 @@
         <v>45855</v>
       </c>
       <c r="B1817">
-        <v>15.8588</v>
+        <v>15.8607</v>
       </c>
       <c r="C1817">
         <v>1.6639999999999999</v>
@@ -53738,7 +53771,7 @@
         <v>45856</v>
       </c>
       <c r="B1818">
-        <v>16.158000000000001</v>
+        <v>16.1599</v>
       </c>
       <c r="C1818">
         <v>1.6679999999999999</v>
@@ -53756,7 +53789,7 @@
         <v>45857</v>
       </c>
       <c r="B1819">
-        <v>16.148199999999999</v>
+        <v>16.150099999999998</v>
       </c>
       <c r="C1819">
         <v>1.6679999999999999</v>
@@ -53774,7 +53807,7 @@
         <v>45858</v>
       </c>
       <c r="B1820">
-        <v>16.168099999999999</v>
+        <v>16.170100000000001</v>
       </c>
       <c r="C1820">
         <v>1.6679999999999999</v>
@@ -53792,7 +53825,7 @@
         <v>45859</v>
       </c>
       <c r="B1821">
-        <v>16.315000000000001</v>
+        <v>16.317</v>
       </c>
       <c r="C1821">
         <v>1.6779999999999999</v>
@@ -53810,7 +53843,7 @@
         <v>45860</v>
       </c>
       <c r="B1822">
-        <v>16.3858</v>
+        <v>16.387599999999999</v>
       </c>
       <c r="C1822">
         <v>1.694</v>
@@ -53828,7 +53861,7 @@
         <v>45861</v>
       </c>
       <c r="B1823">
-        <v>16.7972</v>
+        <v>16.799099999999999</v>
       </c>
       <c r="C1823">
         <v>1.708</v>
@@ -53846,7 +53879,7 @@
         <v>45862</v>
       </c>
       <c r="B1824">
-        <v>16.834499999999998</v>
+        <v>16.836400000000001</v>
       </c>
       <c r="C1824">
         <v>1.742</v>
@@ -53864,7 +53897,7 @@
         <v>45863</v>
       </c>
       <c r="B1825">
-        <v>16.650099999999998</v>
+        <v>16.652000000000001</v>
       </c>
       <c r="C1825">
         <v>1.7390000000000001</v>
@@ -53882,7 +53915,7 @@
         <v>45864</v>
       </c>
       <c r="B1826">
-        <v>16.6389</v>
+        <v>16.640799999999999</v>
       </c>
       <c r="C1826">
         <v>1.7390000000000001</v>
@@ -53900,7 +53933,7 @@
         <v>45865</v>
       </c>
       <c r="B1827">
-        <v>16.6312</v>
+        <v>16.633099999999999</v>
       </c>
       <c r="C1827">
         <v>1.7390000000000001</v>
@@ -53918,7 +53951,7 @@
         <v>45866</v>
       </c>
       <c r="B1828">
-        <v>16.61</v>
+        <v>16.611899999999999</v>
       </c>
       <c r="C1828">
         <v>1.7190000000000001</v>
@@ -53936,7 +53969,7 @@
         <v>45867</v>
       </c>
       <c r="B1829">
-        <v>16.5487</v>
+        <v>16.550599999999999</v>
       </c>
       <c r="C1829">
         <v>1.748</v>
@@ -53954,7 +53987,7 @@
         <v>45868</v>
       </c>
       <c r="B1830">
-        <v>16.113</v>
+        <v>16.114799999999999</v>
       </c>
       <c r="C1830">
         <v>1.728</v>
@@ -53972,7 +54005,7 @@
         <v>45869</v>
       </c>
       <c r="B1831">
-        <v>15.9877</v>
+        <v>15.9895</v>
       </c>
       <c r="C1831">
         <v>1.712</v>
@@ -53990,7 +54023,7 @@
         <v>45870</v>
       </c>
       <c r="B1832">
-        <v>15.784599999999999</v>
+        <v>15.7864</v>
       </c>
       <c r="C1832">
         <v>1.706</v>
@@ -54008,7 +54041,7 @@
         <v>45871</v>
       </c>
       <c r="B1833">
-        <v>15.773400000000001</v>
+        <v>15.7752</v>
       </c>
       <c r="C1833">
         <v>1.706</v>
@@ -54026,7 +54059,7 @@
         <v>45872</v>
       </c>
       <c r="B1834">
-        <v>15.770200000000001</v>
+        <v>15.772</v>
       </c>
       <c r="C1834">
         <v>1.706</v>
@@ -54044,7 +54077,7 @@
         <v>45873</v>
       </c>
       <c r="B1835">
-        <v>15.981299999999999</v>
+        <v>15.9832</v>
       </c>
       <c r="C1835">
         <v>1.7110000000000001</v>
@@ -54062,7 +54095,7 @@
         <v>45874</v>
       </c>
       <c r="B1836">
-        <v>16.122599999999998</v>
+        <v>16.124500000000001</v>
       </c>
       <c r="C1836">
         <v>1.712</v>
@@ -54080,7 +54113,7 @@
         <v>45875</v>
       </c>
       <c r="B1837">
-        <v>16.126100000000001</v>
+        <v>16.128299999999999</v>
       </c>
       <c r="C1837">
         <v>1.704</v>
@@ -54098,7 +54131,7 @@
         <v>45876</v>
       </c>
       <c r="B1838">
-        <v>16.1707</v>
+        <v>16.1724</v>
       </c>
       <c r="C1838">
         <v>1.698</v>
@@ -54116,7 +54149,7 @@
         <v>45877</v>
       </c>
       <c r="B1839">
-        <v>15.922599999999999</v>
+        <v>15.923999999999999</v>
       </c>
       <c r="C1839">
         <v>1.6990000000000001</v>
@@ -54134,7 +54167,7 @@
         <v>45878</v>
       </c>
       <c r="B1840">
-        <v>15.9123</v>
+        <v>15.9137</v>
       </c>
       <c r="C1840">
         <v>1.6990000000000001</v>
@@ -54152,7 +54185,7 @@
         <v>45879</v>
       </c>
       <c r="B1841">
-        <v>15.894299999999999</v>
+        <v>15.8957</v>
       </c>
       <c r="C1841">
         <v>1.6990000000000001</v>
@@ -54170,7 +54203,7 @@
         <v>45880</v>
       </c>
       <c r="B1842">
-        <v>15.904199999999999</v>
+        <v>15.9056</v>
       </c>
       <c r="C1842">
         <v>1.7230000000000001</v>
@@ -54188,7 +54221,7 @@
         <v>45881</v>
       </c>
       <c r="B1843">
-        <v>15.8239</v>
+        <v>15.8253</v>
       </c>
       <c r="C1843">
         <v>1.7310000000000001</v>
@@ -54206,7 +54239,7 @@
         <v>45882</v>
       </c>
       <c r="B1844">
-        <v>16.369399999999999</v>
+        <v>16.370899999999999</v>
       </c>
       <c r="C1844">
         <v>1.7270000000000001</v>
@@ -54224,7 +54257,7 @@
         <v>45883</v>
       </c>
       <c r="B1845">
-        <v>16.218699999999998</v>
+        <v>16.220099999999999</v>
       </c>
       <c r="C1845">
         <v>1.738</v>
@@ -54242,7 +54275,7 @@
         <v>45884</v>
       </c>
       <c r="B1846">
-        <v>16.142600000000002</v>
+        <v>16.144100000000002</v>
       </c>
       <c r="C1846">
         <v>1.748</v>
@@ -54260,7 +54293,7 @@
         <v>45885</v>
       </c>
       <c r="B1847">
-        <v>16.135000000000002</v>
+        <v>16.136500000000002</v>
       </c>
       <c r="C1847">
         <v>1.748</v>
@@ -54278,7 +54311,7 @@
         <v>45886</v>
       </c>
       <c r="B1848">
-        <v>16.153099999999998</v>
+        <v>16.154599999999999</v>
       </c>
       <c r="C1848">
         <v>1.748</v>
@@ -54296,7 +54329,7 @@
         <v>45887</v>
       </c>
       <c r="B1849">
-        <v>16.2286</v>
+        <v>16.2302</v>
       </c>
       <c r="C1849">
         <v>1.784</v>
@@ -54314,7 +54347,7 @@
         <v>45888</v>
       </c>
       <c r="B1850">
-        <v>16.138999999999999</v>
+        <v>16.1403</v>
       </c>
       <c r="C1850">
         <v>1.7729999999999999</v>
@@ -54332,7 +54365,7 @@
         <v>45889</v>
       </c>
       <c r="B1851">
-        <v>16.1113</v>
+        <v>16.111899999999999</v>
       </c>
       <c r="C1851">
         <v>1.786</v>
@@ -54350,7 +54383,7 @@
         <v>45890</v>
       </c>
       <c r="B1852">
-        <v>16.0047</v>
+        <v>16.005199999999999</v>
       </c>
       <c r="C1852">
         <v>1.7689999999999999</v>
@@ -54368,7 +54401,7 @@
         <v>45891</v>
       </c>
       <c r="B1853">
-        <v>16.444500000000001</v>
+        <v>16.444900000000001</v>
       </c>
       <c r="C1853">
         <v>1.7869999999999999</v>
@@ -54386,7 +54419,7 @@
         <v>45892</v>
       </c>
       <c r="B1854">
-        <v>16.431899999999999</v>
+        <v>16.432300000000001</v>
       </c>
       <c r="C1854">
         <v>1.7869999999999999</v>
@@ -54404,7 +54437,7 @@
         <v>45893</v>
       </c>
       <c r="B1855">
-        <v>16.410900000000002</v>
+        <v>16.411200000000001</v>
       </c>
       <c r="C1855">
         <v>1.7869999999999999</v>
@@ -54422,7 +54455,7 @@
         <v>45894</v>
       </c>
       <c r="B1856">
-        <v>16.8995</v>
+        <v>16.897099999999998</v>
       </c>
       <c r="C1856">
         <v>1.7669999999999999</v>
@@ -54440,7 +54473,7 @@
         <v>45895</v>
       </c>
       <c r="B1857">
-        <v>16.767900000000001</v>
+        <v>16.7654</v>
       </c>
       <c r="C1857">
         <v>1.768</v>
@@ -54458,7 +54491,7 @@
         <v>45896</v>
       </c>
       <c r="B1858">
-        <v>16.759899999999998</v>
+        <v>16.760200000000001</v>
       </c>
       <c r="C1858">
         <v>1.77</v>
@@ -54467,7 +54500,7 @@
         <v>4.2343000000000002</v>
       </c>
       <c r="E1858">
-        <f t="shared" ref="E1858:E1871" si="29">C1858-D1858</f>
+        <f t="shared" ref="E1858:E1873" si="29">C1858-D1858</f>
         <v>-2.4643000000000002</v>
       </c>
     </row>
@@ -54476,7 +54509,7 @@
         <v>45897</v>
       </c>
       <c r="B1859">
-        <v>16.8978</v>
+        <v>16.889199999999999</v>
       </c>
       <c r="C1859">
         <v>1.792</v>
@@ -54494,7 +54527,7 @@
         <v>45898</v>
       </c>
       <c r="B1860">
-        <v>17.1873</v>
+        <v>17.1784</v>
       </c>
       <c r="C1860">
         <v>1.786</v>
@@ -54512,7 +54545,7 @@
         <v>45899</v>
       </c>
       <c r="B1861">
-        <v>17.195900000000002</v>
+        <v>17.186900000000001</v>
       </c>
       <c r="C1861">
         <v>1.786</v>
@@ -54530,7 +54563,7 @@
         <v>45900</v>
       </c>
       <c r="B1862">
-        <v>17.334099999999999</v>
+        <v>17.327100000000002</v>
       </c>
       <c r="C1862">
         <v>1.786</v>
@@ -54548,7 +54581,7 @@
         <v>45901</v>
       </c>
       <c r="B1863">
-        <v>17.810300000000002</v>
+        <v>17.802199999999999</v>
       </c>
       <c r="C1863">
         <v>1.7809999999999999</v>
@@ -54566,7 +54599,7 @@
         <v>45902</v>
       </c>
       <c r="B1864">
-        <v>17.7315</v>
+        <v>17.722899999999999</v>
       </c>
       <c r="C1864">
         <v>1.772</v>
@@ -54584,7 +54617,7 @@
         <v>45903</v>
       </c>
       <c r="B1865">
-        <v>17.593699999999998</v>
+        <v>17.585100000000001</v>
       </c>
       <c r="C1865">
         <v>1.7509999999999999</v>
@@ -54602,7 +54635,7 @@
         <v>45904</v>
       </c>
       <c r="B1866">
-        <v>17.2821</v>
+        <v>17.273399999999999</v>
       </c>
       <c r="C1866">
         <v>1.7569999999999999</v>
@@ -54620,7 +54653,7 @@
         <v>45905</v>
       </c>
       <c r="B1867">
-        <v>17.639800000000001</v>
+        <v>17.630800000000001</v>
       </c>
       <c r="C1867">
         <v>1.776</v>
@@ -54638,7 +54671,7 @@
         <v>45906</v>
       </c>
       <c r="B1868">
-        <v>17.625900000000001</v>
+        <v>17.616900000000001</v>
       </c>
       <c r="C1868">
         <v>1.776</v>
@@ -54656,7 +54689,7 @@
         <v>45907</v>
       </c>
       <c r="B1869">
-        <v>17.5962</v>
+        <v>17.5871</v>
       </c>
       <c r="C1869">
         <v>1.776</v>
@@ -54674,7 +54707,7 @@
         <v>45908</v>
       </c>
       <c r="B1870">
-        <v>19.401199999999999</v>
+        <v>19.415500000000002</v>
       </c>
       <c r="C1870">
         <v>1.7909999999999999</v>
@@ -54692,7 +54725,7 @@
         <v>45909</v>
       </c>
       <c r="B1871">
-        <v>19.634599999999999</v>
+        <v>19.694099999999999</v>
       </c>
       <c r="C1871">
         <v>1.8009999999999999</v>
@@ -54706,10 +54739,40 @@
       </c>
     </row>
     <row r="1872" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1872" s="1"/>
-    </row>
-    <row r="1873" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A1873" s="1"/>
+      <c r="A1872" s="1">
+        <v>45910</v>
+      </c>
+      <c r="B1872">
+        <v>19.921600000000002</v>
+      </c>
+      <c r="C1872">
+        <v>1.8240000000000001</v>
+      </c>
+      <c r="D1872">
+        <v>4.0453999999999999</v>
+      </c>
+      <c r="E1872">
+        <f t="shared" si="29"/>
+        <v>-2.2214</v>
+      </c>
+    </row>
+    <row r="1873" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1873" s="1">
+        <v>45911</v>
+      </c>
+      <c r="B1873">
+        <v>19.860399999999998</v>
+      </c>
+      <c r="C1873">
+        <v>1.8069999999999999</v>
+      </c>
+      <c r="D1873">
+        <v>4.0034999999999998</v>
+      </c>
+      <c r="E1873">
+        <f t="shared" si="29"/>
+        <v>-2.1964999999999999</v>
+      </c>
     </row>
   </sheetData>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C275">

</xml_diff>